<commit_message>
read env file to populate credentials
</commit_message>
<xml_diff>
--- a/options_analysis/nse_holidays_2026.xlsx
+++ b/options_analysis/nse_holidays_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\chandra\python\Stocks\NSEOptionsStrategy\options_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC39B64-DD69-48DE-B335-55598704DC88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F67313-7504-4D79-8FAE-B2086A3C71AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3703" yWindow="3703" windowWidth="20571" windowHeight="10834" xr2:uid="{01B09D65-F972-4438-A9C1-2ED96EBAC836}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="27634" windowHeight="15034" xr2:uid="{01B09D65-F972-4438-A9C1-2ED96EBAC836}"/>
   </bookViews>
   <sheets>
     <sheet name="nse_holidays_2026" sheetId="1" r:id="rId1"/>
@@ -112,21 +112,15 @@
       <family val="34"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFBFBFB"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -134,86 +128,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFDDDDDD"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFDDDDDD"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFDDDDDD"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFDDDDDD"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFDDDDDD"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFDDDDDD"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFDDDDDD"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,178 +462,178 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A2" s="9">
+      <c r="A2" s="2">
         <v>46048</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A3" s="9">
+      <c r="A3" s="2">
         <v>46084</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A4" s="9">
+      <c r="A4" s="2">
         <v>46107</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A5" s="9">
+      <c r="A5" s="2">
         <v>46112</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A6" s="9">
+      <c r="A6" s="2">
         <v>46115</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A7" s="9">
+      <c r="A7" s="2">
         <v>46126</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A8" s="9">
+      <c r="A8" s="2">
         <v>46143</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A9" s="9">
+      <c r="A9" s="2">
         <v>46170</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A10" s="9">
+      <c r="A10" s="2">
         <v>46199</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A11" s="9">
+      <c r="A11" s="2">
         <v>46279</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A12" s="9">
+      <c r="A12" s="2">
         <v>46297</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A13" s="9">
+      <c r="A13" s="2">
         <v>46315</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A14" s="9">
+      <c r="A14" s="2">
         <v>46336</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A15" s="9">
+      <c r="A15" s="2">
         <v>46350</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A16" s="9">
+      <c r="A16" s="2">
         <v>46381</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="3" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>